<commit_message>
refinements, github actions, & fixes
</commit_message>
<xml_diff>
--- a/data/KPI List.xlsx
+++ b/data/KPI List.xlsx
@@ -38,89 +38,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={C5511CA9-58C7-4605-9BB3-9BEA8B419DDC}</author>
-    <author>tc={BD693F1B-01E9-4C4C-9011-25EAAC4D6393}</author>
-    <author>tc={D522731A-081F-4B21-8187-5DB02169B021}</author>
-    <author>tc={8BEF53BB-CA65-4CEB-8A25-2357D244AB9C}</author>
-    <author>tc={326222E1-34BF-4AF1-8734-24B0260EB0E3}</author>
-    <author>tc={3882223C-4C38-4294-BC32-EB5330619167}</author>
-    <author>tc={63625332-174C-41FC-ACB2-78BBEBD56086}</author>
-    <author>tc={BBF9D816-0F3D-46FC-959C-4942317A7C7D}</author>
-  </authors>
-  <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{C5511CA9-58C7-4605-9BB3-9BEA8B419DDC}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Higher level KPIs using this KPI as data source</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{BD693F1B-01E9-4C4C-9011-25EAAC4D6393}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Represents the hierarchy level of the KPI in the system. 0 being the highest level indicator.
-Reply:
-    Wird irgendwo deutlich welche Tier 2 in welche Tier 1 KPI einfließen?</t>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="2" shapeId="0" xr:uid="{D522731A-081F-4B21-8187-5DB02169B021}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    This is the ID for automating the calculation.</t>
-      </text>
-    </comment>
-    <comment ref="C36" authorId="3" shapeId="0" xr:uid="{8BEF53BB-CA65-4CEB-8A25-2357D244AB9C}">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Die Gehälter und Löhne der Mitarbeiter, die direkt an der Produktion beteiligt sind </t>
-      </text>
-    </comment>
-    <comment ref="C37" authorId="4" shapeId="0" xr:uid="{326222E1-34BF-4AF1-8734-24B0260EB0E3}">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Kosten, die indirekt mit der Produktion zusammenhängen, wie z.B. Miete, Strom, Abschreibung von Produktionsanlagen, Wartung und Betriebsmittel </t>
-      </text>
-    </comment>
-    <comment ref="C38" authorId="5" shapeId="0" xr:uid="{3882223C-4C38-4294-BC32-EB5330619167}">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Die Kosten für die Verpackung, wenn diese für den Verkauf des Produkts erforderlich ist </t>
-      </text>
-    </comment>
-    <comment ref="C39" authorId="6" shapeId="0" xr:uid="{63625332-174C-41FC-ACB2-78BBEBD56086}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Die Kosten für den Transport der hergestellten Waren zum Lager des Unternehmens</t>
-      </text>
-    </comment>
-    <comment ref="C40" authorId="7" shapeId="0" xr:uid="{BBF9D816-0F3D-46FC-959C-4942317A7C7D}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Die Kosten für den Transport der hergestellten Waren zum Lager des Unternehmens</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11045,14 +10962,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Reviewer 1" id="{499600EE-6151-4467-A996-F0CDCF878DCE}" providerId="None"/>
-  <person displayName="Hutomo Saleh" id="{83A7B59B-F170-4A61-B7A7-FAE8F7A9C5A1}" providerId="None"/>
-  <person displayName="Reviewer 2" id="{1812CDE6-FC44-4115-8725-B11009A6CF17}" providerId="None"/>
-</personList>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{BB4FB320-0019-488D-9587-D7A4F3CC6C06}" name="Tabelle4" displayName="Tabelle4" ref="B5:C10" totalsRowShown="0" headerRowDxfId="135" dataDxfId="133" headerRowBorderDxfId="134" tableBorderDxfId="132">
   <autoFilter ref="B5:C10" xr:uid="{BB4FB320-0019-488D-9587-D7A4F3CC6C06}"/>
@@ -11527,38 +11436,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F1" dT="2025-05-20T09:22:26.02" personId="{1812CDE6-FC44-4115-8725-B11009A6CF17}" id="{C5511CA9-58C7-4605-9BB3-9BEA8B419DDC}">
-    <text>Higher level KPIs using this KPI as data source</text>
-  </threadedComment>
-  <threadedComment ref="K1" dT="2025-05-06T09:07:50.08" personId="{83A7B59B-F170-4A61-B7A7-FAE8F7A9C5A1}" id="{BD693F1B-01E9-4C4C-9011-25EAAC4D6393}">
-    <text>Represents the hierarchy level of the KPI in the system. 0 being the highest level indicator.</text>
-  </threadedComment>
-  <threadedComment ref="K1" dT="2025-05-08T12:11:47.94" personId="{499600EE-6151-4467-A996-F0CDCF878DCE}" id="{131E788D-B644-41EC-A1BB-863D24050313}" parentId="{BD693F1B-01E9-4C4C-9011-25EAAC4D6393}">
-    <text>Wird irgendwo deutlich welche Tier 2 in welche Tier 1 KPI einfließen?</text>
-  </threadedComment>
-  <threadedComment ref="O1" dT="2026-02-03T08:39:31.85" personId="{83A7B59B-F170-4A61-B7A7-FAE8F7A9C5A1}" id="{D522731A-081F-4B21-8187-5DB02169B021}">
-    <text>This is the ID for automating the calculation.</text>
-  </threadedComment>
-  <threadedComment ref="C36" dT="2025-06-17T14:23:40.43" personId="{1812CDE6-FC44-4115-8725-B11009A6CF17}" id="{8BEF53BB-CA65-4CEB-8A25-2357D244AB9C}">
-    <text xml:space="preserve">Die Gehälter und Löhne der Mitarbeiter, die direkt an der Produktion beteiligt sind </text>
-  </threadedComment>
-  <threadedComment ref="C37" dT="2025-06-17T14:23:50.78" personId="{1812CDE6-FC44-4115-8725-B11009A6CF17}" id="{326222E1-34BF-4AF1-8734-24B0260EB0E3}">
-    <text xml:space="preserve">Kosten, die indirekt mit der Produktion zusammenhängen, wie z.B. Miete, Strom, Abschreibung von Produktionsanlagen, Wartung und Betriebsmittel </text>
-  </threadedComment>
-  <threadedComment ref="C38" dT="2025-06-17T14:24:02.59" personId="{1812CDE6-FC44-4115-8725-B11009A6CF17}" id="{3882223C-4C38-4294-BC32-EB5330619167}">
-    <text xml:space="preserve">Die Kosten für die Verpackung, wenn diese für den Verkauf des Produkts erforderlich ist </text>
-  </threadedComment>
-  <threadedComment ref="C39" dT="2025-06-17T14:24:18.40" personId="{1812CDE6-FC44-4115-8725-B11009A6CF17}" id="{63625332-174C-41FC-ACB2-78BBEBD56086}">
-    <text>Die Kosten für den Transport der hergestellten Waren zum Lager des Unternehmens</text>
-  </threadedComment>
-  <threadedComment ref="C40" dT="2025-06-17T14:24:18.40" personId="{1812CDE6-FC44-4115-8725-B11009A6CF17}" id="{BBF9D816-0F3D-46FC-959C-4942317A7C7D}">
-    <text>Die Kosten für den Transport der hergestellten Waren zum Lager des Unternehmens</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718D9E52-D5F2-47DF-95F4-841388F8B6B3}">
   <sheetPr>
@@ -33999,7 +33876,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
-  <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
     <tablePart r:id="rId3"/>
   </tableParts>

</xml_diff>